<commit_message>
Cuello Cerrado de fábrica, sin hoodie, moldes en blanco (quitan el rasgo), cinto sin hebilla
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5ByHgyXpZwXMUmHLQD8vD
</commit_message>
<xml_diff>
--- a/docs/recetas_moldes_propuesta.xlsx
+++ b/docs/recetas_moldes_propuesta.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="347">
   <si>
     <t xml:space="preserve">Ítems en blanco — recetas con forma (letras en la hoja Leyenda)</t>
   </si>
@@ -298,12 +298,6 @@
     <t xml:space="preserve">modamod:molde_calce_ajustado</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Calce: Normal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_calce_normal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Calce: Suelto</t>
   </si>
   <si>
@@ -319,12 +313,6 @@
     <t xml:space="preserve">Ruedo</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Ruedo: Recto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_ruedo_recto</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Ruedo: Ajustado</t>
   </si>
   <si>
@@ -364,12 +352,6 @@
     <t xml:space="preserve">Pollera</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Pollera: Campana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_pollera_campana</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Pollera: Tableada</t>
   </si>
   <si>
@@ -412,12 +394,6 @@
     <t xml:space="preserve">Delantal</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Delantal: Recto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_delantal_recto</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Delantal: Trapecio</t>
   </si>
   <si>
@@ -442,12 +418,6 @@
     <t xml:space="preserve">modamod:molde_delantal_feston</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Delantal: Tirantes: Sin tirantes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_delantal_tirantes_sin</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Delantal: Tirantes: Rectos</t>
   </si>
   <si>
@@ -460,12 +430,6 @@
     <t xml:space="preserve">modamod:molde_delantal_tirantes_cruzados</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Delantal: Cobertura: Envolvente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_delantal_cobertura_envolvente</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Delantal: Cobertura: Solo el frente</t>
   </si>
   <si>
@@ -481,12 +445,6 @@
     <t xml:space="preserve">Capa</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Capa: Ruedo recto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_ruedo_recto</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Capa: Ruedo redondeado</t>
   </si>
   <si>
@@ -505,30 +463,12 @@
     <t xml:space="preserve">modamod:molde_capa_cuello_alto</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Capa: Sin cuello</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_sin_cuello</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Capa: Con capucha</t>
   </si>
   <si>
     <t xml:space="preserve">modamod:molde_capa_con_capucha</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Capa: Sin capucha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_sin_capucha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molde de Capa: Sin embozo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_embozo_ninguno</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Capa: Borde del embozo</t>
   </si>
   <si>
@@ -538,21 +478,9 @@
     <t xml:space="preserve">Cuero</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Capa: Sin borde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_borde_ninguno</t>
-  </si>
-  <si>
     <t xml:space="preserve">Remera (frente, capucha, solapa)</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Chaqueta: Frente cerrado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_chaqueta_frente_cerrada</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Chaqueta: Frente abierto</t>
   </si>
   <si>
@@ -577,18 +505,6 @@
     <t xml:space="preserve">modamod:molde_chaqueta_capucha_con</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Chaqueta: Sin capucha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_chaqueta_capucha_sin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molde de Chaqueta: Sin solapas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_chaqueta_solapa_ninguna</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Chaqueta: Solapas en pico</t>
   </si>
   <si>
@@ -610,12 +526,6 @@
     <t xml:space="preserve">Sombrero</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Sombrero: Ala ancha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_sombrero_ala_ancha</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Sombrero: Ala corta</t>
   </si>
   <si>
@@ -634,12 +544,6 @@
     <t xml:space="preserve">modamod:molde_sombrero_ala_cofia</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Sombrero: Punta recta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_sombrero_punta_recta</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Sombrero: Punta doblada</t>
   </si>
   <si>
@@ -667,24 +571,12 @@
     <t xml:space="preserve">modamod:molde_banda_ancho_fino</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Banda: Ancho medio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_banda_ancho_medio</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Banda: Ancho grande</t>
   </si>
   <si>
     <t xml:space="preserve">modamod:molde_banda_ancho_ancho</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Banda: Sin herraje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_banda_herraje_ninguno</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Banda: Herraje placa</t>
   </si>
   <si>
@@ -739,24 +631,12 @@
     <t xml:space="preserve">modamod:molde_borcego_cana_baja</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Borcegos: Caña media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_borcego_cana_media</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Borcegos: Caña alta</t>
   </si>
   <si>
     <t xml:space="preserve">modamod:molde_borcego_cana_alta</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Borcegos: Suela chata</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_borcego_suela_chata</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Borcegos: Suela de plataforma</t>
   </si>
   <si>
@@ -766,12 +646,6 @@
     <t xml:space="preserve">Bola de slime</t>
   </si>
   <si>
-    <t xml:space="preserve">Molde de Borcegos: Botamanga por dentro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_borcego_botamanga_adentro</t>
-  </si>
-  <si>
     <t xml:space="preserve">Molde de Borcegos: Botamanga por fuera</t>
   </si>
   <si>
@@ -781,12 +655,6 @@
     <t xml:space="preserve">Trama</t>
   </si>
   <si>
-    <t xml:space="preserve">Trama: Lisa (sin trama)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_red_lisa</t>
-  </si>
-  <si>
     <t xml:space="preserve">Trama: Fina</t>
   </si>
   <si>
@@ -1049,6 +917,9 @@
   </si>
   <si>
     <t xml:space="preserve">No están: el molde de mangas y el de cuello de capucha (jubilados) ni las plantillas personalizadas (solo creativo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ya no hay molde de cuello de capucha ni 'Molde de mangas' (jubilados): no están en la lista.</t>
   </si>
   <si>
     <t xml:space="preserve">Decisiones pendientes</t>
@@ -2024,7 +1895,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N150"/>
+  <dimension ref="A1:N129"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -2706,7 +2577,7 @@
         <v>60</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23" s="12"/>
       <c r="J23" s="7"/>
@@ -2715,7 +2586,7 @@
       </c>
       <c r="L23" s="8" t="n">
         <f aca="false">1+SUM(F23,H23,J23)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M23" s="8" t="str">
         <f aca="false">IF(L23&gt;9,"¡más de 9!","ok")</f>
@@ -2742,7 +2613,7 @@
         <v>60</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I24" s="12"/>
       <c r="J24" s="7"/>
@@ -2751,7 +2622,7 @@
       </c>
       <c r="L24" s="8" t="n">
         <f aca="false">1+SUM(F24,H24,J24)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M24" s="8" t="str">
         <f aca="false">IF(L24&gt;9,"¡más de 9!","ok")</f>
@@ -2759,58 +2630,58 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="5" t="s">
+      <c r="A25" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
+      <c r="L25" s="10"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D25" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="H25" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I25" s="12"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L25" s="8" t="n">
-        <f aca="false">1+SUM(F25,H25,J25)</f>
-        <v>7</v>
-      </c>
-      <c r="M25" s="8" t="str">
-        <f aca="false">IF(L25&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+      <c r="C26" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
+      <c r="D26" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="12"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" s="8" t="n">
+        <f aca="false">1+SUM(F26,H26,J26)</f>
+        <v>3</v>
+      </c>
+      <c r="M26" s="8" t="str">
+        <f aca="false">IF(L26&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
@@ -2828,8 +2699,12 @@
       <c r="F27" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G27" s="12"/>
-      <c r="H27" s="7"/>
+      <c r="G27" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I27" s="12"/>
       <c r="J27" s="7"/>
       <c r="K27" s="7" t="n">
@@ -2837,7 +2712,7 @@
       </c>
       <c r="L27" s="8" t="n">
         <f aca="false">1+SUM(F27,H27,J27)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M27" s="8" t="str">
         <f aca="false">IF(L27&gt;9,"¡más de 9!","ok")</f>
@@ -2861,7 +2736,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="H28" s="7" t="n">
         <v>1</v>
@@ -2882,10 +2757,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D29" s="12" t="s">
         <v>17</v>
@@ -2897,7 +2772,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="H29" s="7" t="n">
         <v>1</v>
@@ -2918,10 +2793,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>17</v>
@@ -2933,7 +2808,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="H30" s="7" t="n">
         <v>1</v>
@@ -2953,48 +2828,30 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C31" s="11" t="s">
+      <c r="A31" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="D31" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E31" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="H31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I31" s="12"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" s="8" t="n">
-        <f aca="false">1+SUM(F31,H31,J31)</f>
-        <v>3</v>
-      </c>
-      <c r="M31" s="8" t="str">
-        <f aca="false">IF(L31&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C32" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="11" t="s">
-        <v>111</v>
-      </c>
       <c r="D32" s="12" t="s">
         <v>17</v>
       </c>
@@ -3005,10 +2862,10 @@
         <v>1</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I32" s="12"/>
       <c r="J32" s="7"/>
@@ -3017,7 +2874,7 @@
       </c>
       <c r="L32" s="8" t="n">
         <f aca="false">1+SUM(F32,H32,J32)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M32" s="8" t="str">
         <f aca="false">IF(L32&gt;9,"¡más de 9!","ok")</f>
@@ -3025,22 +2882,40 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="s">
+      <c r="B33" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C33" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="10"/>
-      <c r="N33" s="10"/>
+      <c r="D33" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="12"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="8" t="n">
+        <f aca="false">1+SUM(F33,H33,J33)</f>
+        <v>3</v>
+      </c>
+      <c r="M33" s="8" t="str">
+        <f aca="false">IF(L33&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="5" t="s">
@@ -3064,14 +2939,18 @@
       <c r="H34" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I34" s="12"/>
-      <c r="J34" s="7"/>
+      <c r="I34" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L34" s="8" t="n">
         <f aca="false">1+SUM(F34,H34,J34)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M34" s="8" t="str">
         <f aca="false">IF(L34&gt;9,"¡más de 9!","ok")</f>
@@ -3080,10 +2959,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D35" s="12" t="s">
         <v>17</v>
@@ -3098,10 +2977,14 @@
         <v>60</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="I35" s="12"/>
-      <c r="J35" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K35" s="7" t="n">
         <v>1</v>
       </c>
@@ -3116,10 +2999,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>17</v>
@@ -3134,7 +3017,7 @@
         <v>73</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" s="12"/>
       <c r="J36" s="7"/>
@@ -3143,7 +3026,7 @@
       </c>
       <c r="L36" s="8" t="n">
         <f aca="false">1+SUM(F36,H36,J36)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M36" s="8" t="str">
         <f aca="false">IF(L36&gt;9,"¡más de 9!","ok")</f>
@@ -3152,10 +3035,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D37" s="12" t="s">
         <v>17</v>
@@ -3167,13 +3050,13 @@
         <v>1</v>
       </c>
       <c r="G37" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="12" t="s">
         <v>60</v>
-      </c>
-      <c r="H37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I37" s="12" t="s">
-        <v>121</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>1</v>
@@ -3191,51 +3074,29 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="5" t="s">
+      <c r="A38" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="C38" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E38" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="H38" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I38" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="J38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L38" s="8" t="n">
-        <f aca="false">1+SUM(F38,H38,J38)</f>
-        <v>5</v>
-      </c>
-      <c r="M38" s="8" t="str">
-        <f aca="false">IF(L38&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+      <c r="N38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>124</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>125</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>17</v>
@@ -3250,7 +3111,7 @@
         <v>73</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I39" s="12"/>
       <c r="J39" s="7"/>
@@ -3259,7 +3120,7 @@
       </c>
       <c r="L39" s="8" t="n">
         <f aca="false">1+SUM(F39,H39,J39)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M39" s="8" t="str">
         <f aca="false">IF(L39&gt;9,"¡más de 9!","ok")</f>
@@ -3268,11 +3129,11 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="C40" s="11" t="s">
-        <v>127</v>
-      </c>
       <c r="D40" s="12" t="s">
         <v>17</v>
       </c>
@@ -3283,23 +3144,19 @@
         <v>1</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="H40" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I40" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="J40" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="I40" s="12"/>
+      <c r="J40" s="7"/>
       <c r="K40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L40" s="8" t="n">
         <f aca="false">1+SUM(F40,H40,J40)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M40" s="8" t="str">
         <f aca="false">IF(L40&gt;9,"¡más de 9!","ok")</f>
@@ -3307,22 +3164,40 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="s">
+      <c r="B41" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10"/>
-      <c r="I41" s="10"/>
-      <c r="J41" s="10"/>
-      <c r="K41" s="10"/>
-      <c r="L41" s="10"/>
-      <c r="M41" s="10"/>
-      <c r="N41" s="10"/>
+      <c r="D41" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="12"/>
+      <c r="J41" s="7"/>
+      <c r="K41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L41" s="8" t="n">
+        <f aca="false">1+SUM(F41,H41,J41)</f>
+        <v>3</v>
+      </c>
+      <c r="M41" s="8" t="str">
+        <f aca="false">IF(L41&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="5" t="s">
@@ -3340,8 +3215,12 @@
       <c r="F42" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="12"/>
-      <c r="H42" s="7"/>
+      <c r="G42" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="H42" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I42" s="12"/>
       <c r="J42" s="7"/>
       <c r="K42" s="7" t="n">
@@ -3349,7 +3228,7 @@
       </c>
       <c r="L42" s="8" t="n">
         <f aca="false">1+SUM(F42,H42,J42)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M42" s="8" t="str">
         <f aca="false">IF(L42&gt;9,"¡más de 9!","ok")</f>
@@ -3409,10 +3288,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I44" s="12"/>
       <c r="J44" s="7"/>
@@ -3421,7 +3300,7 @@
       </c>
       <c r="L44" s="8" t="n">
         <f aca="false">1+SUM(F44,H44,J44)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M44" s="8" t="str">
         <f aca="false">IF(L44&gt;9,"¡más de 9!","ok")</f>
@@ -3444,12 +3323,8 @@
       <c r="F45" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G45" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H45" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="G45" s="12"/>
+      <c r="H45" s="7"/>
       <c r="I45" s="12"/>
       <c r="J45" s="7"/>
       <c r="K45" s="7" t="n">
@@ -3457,7 +3332,7 @@
       </c>
       <c r="L45" s="8" t="n">
         <f aca="false">1+SUM(F45,H45,J45)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M45" s="8" t="str">
         <f aca="false">IF(L45&gt;9,"¡más de 9!","ok")</f>
@@ -3481,7 +3356,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>109</v>
+        <v>73</v>
       </c>
       <c r="H46" s="7" t="n">
         <v>1</v>
@@ -3501,43 +3376,29 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="5" t="s">
+      <c r="A47" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C47" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="D47" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E47" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" s="12"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L47" s="8" t="n">
-        <f aca="false">1+SUM(F47,H47,J47)</f>
-        <v>2</v>
-      </c>
-      <c r="M47" s="8" t="str">
-        <f aca="false">IF(L47&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="10"/>
+      <c r="K47" s="10"/>
+      <c r="L47" s="10"/>
+      <c r="M47" s="10"/>
+      <c r="N47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C48" s="11" t="s">
         <v>141</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>142</v>
       </c>
       <c r="D48" s="12" t="s">
         <v>17</v>
@@ -3570,11 +3431,11 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C49" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="C49" s="11" t="s">
-        <v>144</v>
-      </c>
       <c r="D49" s="12" t="s">
         <v>17</v>
       </c>
@@ -3585,10 +3446,10 @@
         <v>1</v>
       </c>
       <c r="G49" s="12" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I49" s="12"/>
       <c r="J49" s="7"/>
@@ -3597,7 +3458,7 @@
       </c>
       <c r="L49" s="8" t="n">
         <f aca="false">1+SUM(F49,H49,J49)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M49" s="8" t="str">
         <f aca="false">IF(L49&gt;9,"¡más de 9!","ok")</f>
@@ -3606,10 +3467,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C50" s="11" t="s">
         <v>145</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>146</v>
       </c>
       <c r="D50" s="12" t="s">
         <v>17</v>
@@ -3642,11 +3503,11 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C51" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="C51" s="11" t="s">
-        <v>148</v>
-      </c>
       <c r="D51" s="12" t="s">
         <v>17</v>
       </c>
@@ -3656,8 +3517,12 @@
       <c r="F51" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G51" s="12"/>
-      <c r="H51" s="7"/>
+      <c r="G51" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H51" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="I51" s="12"/>
       <c r="J51" s="7"/>
       <c r="K51" s="7" t="n">
@@ -3665,7 +3530,7 @@
       </c>
       <c r="L51" s="8" t="n">
         <f aca="false">1+SUM(F51,H51,J51)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M51" s="8" t="str">
         <f aca="false">IF(L51&gt;9,"¡más de 9!","ok")</f>
@@ -3674,22 +3539,22 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="C52" s="11" t="s">
+      <c r="D52" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="12" t="s">
         <v>150</v>
-      </c>
-      <c r="D52" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>73</v>
       </c>
       <c r="H52" s="7" t="n">
         <v>1</v>
@@ -3742,8 +3607,12 @@
       <c r="F54" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G54" s="12"/>
-      <c r="H54" s="7"/>
+      <c r="G54" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H54" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I54" s="12"/>
       <c r="J54" s="7"/>
       <c r="K54" s="7" t="n">
@@ -3751,7 +3620,7 @@
       </c>
       <c r="L54" s="8" t="n">
         <f aca="false">1+SUM(F54,H54,J54)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M54" s="8" t="str">
         <f aca="false">IF(L54&gt;9,"¡más de 9!","ok")</f>
@@ -3775,10 +3644,10 @@
         <v>1</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I55" s="12"/>
       <c r="J55" s="7"/>
@@ -3787,7 +3656,7 @@
       </c>
       <c r="L55" s="8" t="n">
         <f aca="false">1+SUM(F55,H55,J55)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M55" s="8" t="str">
         <f aca="false">IF(L55&gt;9,"¡más de 9!","ok")</f>
@@ -3811,7 +3680,7 @@
         <v>1</v>
       </c>
       <c r="G56" s="12" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="H56" s="7" t="n">
         <v>3</v>
@@ -3850,7 +3719,7 @@
         <v>60</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57" s="12"/>
       <c r="J57" s="7"/>
@@ -3859,7 +3728,7 @@
       </c>
       <c r="L57" s="8" t="n">
         <f aca="false">1+SUM(F57,H57,J57)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M57" s="8" t="str">
         <f aca="false">IF(L57&gt;9,"¡más de 9!","ok")</f>
@@ -3882,8 +3751,12 @@
       <c r="F58" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="12"/>
-      <c r="H58" s="7"/>
+      <c r="G58" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H58" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I58" s="12"/>
       <c r="J58" s="7"/>
       <c r="K58" s="7" t="n">
@@ -3891,7 +3764,7 @@
       </c>
       <c r="L58" s="8" t="n">
         <f aca="false">1+SUM(F58,H58,J58)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M58" s="8" t="str">
         <f aca="false">IF(L58&gt;9,"¡más de 9!","ok")</f>
@@ -3915,10 +3788,10 @@
         <v>1</v>
       </c>
       <c r="G59" s="12" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H59" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I59" s="12"/>
       <c r="J59" s="7"/>
@@ -3927,7 +3800,7 @@
       </c>
       <c r="L59" s="8" t="n">
         <f aca="false">1+SUM(F59,H59,J59)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M59" s="8" t="str">
         <f aca="false">IF(L59&gt;9,"¡más de 9!","ok")</f>
@@ -3950,8 +3823,12 @@
       <c r="F60" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G60" s="12"/>
-      <c r="H60" s="7"/>
+      <c r="G60" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H60" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I60" s="12"/>
       <c r="J60" s="7"/>
       <c r="K60" s="7" t="n">
@@ -3959,7 +3836,7 @@
       </c>
       <c r="L60" s="8" t="n">
         <f aca="false">1+SUM(F60,H60,J60)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M60" s="8" t="str">
         <f aca="false">IF(L60&gt;9,"¡más de 9!","ok")</f>
@@ -3967,44 +3844,30 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="5" t="s">
+      <c r="A61" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="C61" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="D61" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E61" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F61" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" s="12"/>
-      <c r="H61" s="7"/>
-      <c r="I61" s="12"/>
-      <c r="J61" s="7"/>
-      <c r="K61" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L61" s="8" t="n">
-        <f aca="false">1+SUM(F61,H61,J61)</f>
-        <v>2</v>
-      </c>
-      <c r="M61" s="8" t="str">
-        <f aca="false">IF(L61&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="10"/>
+      <c r="F61" s="10"/>
+      <c r="G61" s="10"/>
+      <c r="H61" s="10"/>
+      <c r="I61" s="10"/>
+      <c r="J61" s="10"/>
+      <c r="K61" s="10"/>
+      <c r="L61" s="10"/>
+      <c r="M61" s="10"/>
+      <c r="N61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C62" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C62" s="11" t="s">
-        <v>169</v>
-      </c>
       <c r="D62" s="12" t="s">
         <v>17</v>
       </c>
@@ -4015,7 +3878,7 @@
         <v>1</v>
       </c>
       <c r="G62" s="12" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="H62" s="7" t="n">
         <v>1</v>
@@ -4036,10 +3899,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D63" s="12" t="s">
         <v>17</v>
@@ -4050,8 +3913,12 @@
       <c r="F63" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G63" s="12"/>
-      <c r="H63" s="7"/>
+      <c r="G63" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H63" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I63" s="12"/>
       <c r="J63" s="7"/>
       <c r="K63" s="7" t="n">
@@ -4059,7 +3926,7 @@
       </c>
       <c r="L63" s="8" t="n">
         <f aca="false">1+SUM(F63,H63,J63)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M63" s="8" t="str">
         <f aca="false">IF(L63&gt;9,"¡más de 9!","ok")</f>
@@ -4067,30 +3934,48 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="10"/>
-      <c r="J64" s="10"/>
-      <c r="K64" s="10"/>
-      <c r="L64" s="10"/>
-      <c r="M64" s="10"/>
-      <c r="N64" s="10"/>
+      <c r="B64" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C64" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E64" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H64" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I64" s="12"/>
+      <c r="J64" s="7"/>
+      <c r="K64" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L64" s="8" t="n">
+        <f aca="false">1+SUM(F64,H64,J64)</f>
+        <v>3</v>
+      </c>
+      <c r="M64" s="8" t="str">
+        <f aca="false">IF(L64&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="C65" s="11" t="s">
-        <v>175</v>
-      </c>
       <c r="D65" s="12" t="s">
         <v>17</v>
       </c>
@@ -4100,8 +3985,12 @@
       <c r="F65" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G65" s="12"/>
-      <c r="H65" s="7"/>
+      <c r="G65" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H65" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I65" s="12"/>
       <c r="J65" s="7"/>
       <c r="K65" s="7" t="n">
@@ -4109,7 +3998,7 @@
       </c>
       <c r="L65" s="8" t="n">
         <f aca="false">1+SUM(F65,H65,J65)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M65" s="8" t="str">
         <f aca="false">IF(L65&gt;9,"¡más de 9!","ok")</f>
@@ -4117,47 +4006,29 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C66" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="D66" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E66" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F66" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G66" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="H66" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I66" s="12"/>
-      <c r="J66" s="7"/>
-      <c r="K66" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L66" s="8" t="n">
-        <f aca="false">1+SUM(F66,H66,J66)</f>
-        <v>3</v>
-      </c>
-      <c r="M66" s="8" t="str">
-        <f aca="false">IF(L66&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="A66" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="10"/>
+      <c r="E66" s="10"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="10"/>
+      <c r="H66" s="10"/>
+      <c r="I66" s="10"/>
+      <c r="J66" s="10"/>
+      <c r="K66" s="10"/>
+      <c r="L66" s="10"/>
+      <c r="M66" s="10"/>
+      <c r="N66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D67" s="12" t="s">
         <v>17</v>
@@ -4169,10 +4040,10 @@
         <v>1</v>
       </c>
       <c r="G67" s="12" t="s">
-        <v>69</v>
+        <v>150</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I67" s="12"/>
       <c r="J67" s="7"/>
@@ -4181,7 +4052,7 @@
       </c>
       <c r="L67" s="8" t="n">
         <f aca="false">1+SUM(F67,H67,J67)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M67" s="8" t="str">
         <f aca="false">IF(L67&gt;9,"¡más de 9!","ok")</f>
@@ -4190,10 +4061,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D68" s="12" t="s">
         <v>17</v>
@@ -4205,10 +4076,10 @@
         <v>1</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I68" s="12"/>
       <c r="J68" s="7"/>
@@ -4217,7 +4088,7 @@
       </c>
       <c r="L68" s="8" t="n">
         <f aca="false">1+SUM(F68,H68,J68)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M68" s="8" t="str">
         <f aca="false">IF(L68&gt;9,"¡más de 9!","ok")</f>
@@ -4226,10 +4097,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C69" s="11" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D69" s="12" t="s">
         <v>17</v>
@@ -4241,10 +4112,10 @@
         <v>1</v>
       </c>
       <c r="G69" s="12" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I69" s="12"/>
       <c r="J69" s="7"/>
@@ -4253,7 +4124,7 @@
       </c>
       <c r="L69" s="8" t="n">
         <f aca="false">1+SUM(F69,H69,J69)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M69" s="8" t="str">
         <f aca="false">IF(L69&gt;9,"¡más de 9!","ok")</f>
@@ -4262,10 +4133,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>17</v>
@@ -4276,8 +4147,12 @@
       <c r="F70" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G70" s="12"/>
-      <c r="H70" s="7"/>
+      <c r="G70" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="H70" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="I70" s="12"/>
       <c r="J70" s="7"/>
       <c r="K70" s="7" t="n">
@@ -4285,7 +4160,7 @@
       </c>
       <c r="L70" s="8" t="n">
         <f aca="false">1+SUM(F70,H70,J70)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M70" s="8" t="str">
         <f aca="false">IF(L70&gt;9,"¡más de 9!","ok")</f>
@@ -4294,22 +4169,26 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F71" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="C71" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="D71" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E71" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F71" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="12"/>
-      <c r="H71" s="7"/>
+      <c r="H71" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I71" s="12"/>
       <c r="J71" s="7"/>
       <c r="K71" s="7" t="n">
@@ -4317,7 +4196,7 @@
       </c>
       <c r="L71" s="8" t="n">
         <f aca="false">1+SUM(F71,H71,J71)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M71" s="8" t="str">
         <f aca="false">IF(L71&gt;9,"¡más de 9!","ok")</f>
@@ -4326,10 +4205,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C72" s="11" t="s">
         <v>188</v>
-      </c>
-      <c r="C72" s="11" t="s">
-        <v>189</v>
       </c>
       <c r="D72" s="12" t="s">
         <v>17</v>
@@ -4362,11 +4241,11 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C73" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="C73" s="11" t="s">
-        <v>191</v>
-      </c>
       <c r="D73" s="12" t="s">
         <v>17</v>
       </c>
@@ -4377,10 +4256,10 @@
         <v>1</v>
       </c>
       <c r="G73" s="12" t="s">
-        <v>73</v>
+        <v>105</v>
       </c>
       <c r="H73" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I73" s="12"/>
       <c r="J73" s="7"/>
@@ -4389,7 +4268,7 @@
       </c>
       <c r="L73" s="8" t="n">
         <f aca="false">1+SUM(F73,H73,J73)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M73" s="8" t="str">
         <f aca="false">IF(L73&gt;9,"¡más de 9!","ok")</f>
@@ -4398,22 +4277,22 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C74" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="C74" s="11" t="s">
+      <c r="D74" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E74" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="12" t="s">
         <v>193</v>
-      </c>
-      <c r="D74" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E74" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F74" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G74" s="12" t="s">
-        <v>60</v>
       </c>
       <c r="H74" s="7" t="n">
         <v>1</v>
@@ -4433,29 +4312,47 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="9" t="s">
+      <c r="B75" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="B75" s="10"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="10"/>
-      <c r="E75" s="10"/>
-      <c r="F75" s="10"/>
-      <c r="G75" s="10"/>
-      <c r="H75" s="10"/>
-      <c r="I75" s="10"/>
-      <c r="J75" s="10"/>
-      <c r="K75" s="10"/>
-      <c r="L75" s="10"/>
-      <c r="M75" s="10"/>
-      <c r="N75" s="10"/>
+      <c r="C75" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="D75" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E75" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F75" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H75" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" s="12"/>
+      <c r="J75" s="7"/>
+      <c r="K75" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L75" s="8" t="n">
+        <f aca="false">1+SUM(F75,H75,J75)</f>
+        <v>3</v>
+      </c>
+      <c r="M75" s="8" t="str">
+        <f aca="false">IF(L75&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D76" s="12" t="s">
         <v>17</v>
@@ -4467,10 +4364,10 @@
         <v>1</v>
       </c>
       <c r="G76" s="12" t="s">
-        <v>170</v>
+        <v>198</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I76" s="12"/>
       <c r="J76" s="7"/>
@@ -4479,7 +4376,7 @@
       </c>
       <c r="L76" s="8" t="n">
         <f aca="false">1+SUM(F76,H76,J76)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M76" s="8" t="str">
         <f aca="false">IF(L76&gt;9,"¡más de 9!","ok")</f>
@@ -4487,47 +4384,29 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B77" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="C77" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="D77" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E77" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F77" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G77" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H77" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I77" s="12"/>
-      <c r="J77" s="7"/>
-      <c r="K77" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L77" s="8" t="n">
-        <f aca="false">1+SUM(F77,H77,J77)</f>
-        <v>3</v>
-      </c>
-      <c r="M77" s="8" t="str">
-        <f aca="false">IF(L77&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="A77" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="10"/>
+      <c r="E77" s="10"/>
+      <c r="F77" s="10"/>
+      <c r="G77" s="10"/>
+      <c r="H77" s="10"/>
+      <c r="I77" s="10"/>
+      <c r="J77" s="10"/>
+      <c r="K77" s="10"/>
+      <c r="L77" s="10"/>
+      <c r="M77" s="10"/>
+      <c r="N77" s="10"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D78" s="12" t="s">
         <v>17</v>
@@ -4539,7 +4418,7 @@
         <v>1</v>
       </c>
       <c r="G78" s="12" t="s">
-        <v>73</v>
+        <v>150</v>
       </c>
       <c r="H78" s="7" t="n">
         <v>1</v>
@@ -4560,10 +4439,10 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D79" s="12" t="s">
         <v>17</v>
@@ -4575,10 +4454,10 @@
         <v>1</v>
       </c>
       <c r="G79" s="12" t="s">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="H79" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79" s="12"/>
       <c r="J79" s="7"/>
@@ -4587,7 +4466,7 @@
       </c>
       <c r="L79" s="8" t="n">
         <f aca="false">1+SUM(F79,H79,J79)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M79" s="8" t="str">
         <f aca="false">IF(L79&gt;9,"¡más de 9!","ok")</f>
@@ -4596,10 +4475,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D80" s="12" t="s">
         <v>17</v>
@@ -4611,19 +4490,23 @@
         <v>1</v>
       </c>
       <c r="G80" s="12" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="H80" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I80" s="12"/>
-      <c r="J80" s="7"/>
+      <c r="I80" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="J80" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K80" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L80" s="8" t="n">
         <f aca="false">1+SUM(F80,H80,J80)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M80" s="8" t="str">
         <f aca="false">IF(L80&gt;9,"¡más de 9!","ok")</f>
@@ -4632,10 +4515,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D81" s="12" t="s">
         <v>17</v>
@@ -4650,7 +4533,7 @@
         <v>73</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I81" s="12"/>
       <c r="J81" s="7"/>
@@ -4659,7 +4542,7 @@
       </c>
       <c r="L81" s="8" t="n">
         <f aca="false">1+SUM(F81,H81,J81)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M81" s="8" t="str">
         <f aca="false">IF(L81&gt;9,"¡más de 9!","ok")</f>
@@ -4668,7 +4551,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B82" s="10"/>
       <c r="C82" s="10"/>
@@ -4686,26 +4569,22 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E83" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F83" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G83" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H83" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="G83" s="12"/>
+      <c r="H83" s="7"/>
       <c r="I83" s="12"/>
       <c r="J83" s="7"/>
       <c r="K83" s="7" t="n">
@@ -4713,7 +4592,7 @@
       </c>
       <c r="L83" s="8" t="n">
         <f aca="false">1+SUM(F83,H83,J83)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M83" s="8" t="str">
         <f aca="false">IF(L83&gt;9,"¡más de 9!","ok")</f>
@@ -4722,26 +4601,22 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C84" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E84" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F84" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H84" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G84" s="12"/>
+      <c r="H84" s="7"/>
       <c r="I84" s="12"/>
       <c r="J84" s="7"/>
       <c r="K84" s="7" t="n">
@@ -4749,7 +4624,7 @@
       </c>
       <c r="L84" s="8" t="n">
         <f aca="false">1+SUM(F84,H84,J84)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M84" s="8" t="str">
         <f aca="false">IF(L84&gt;9,"¡más de 9!","ok")</f>
@@ -4758,22 +4633,22 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C85" s="11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D85" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E85" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F85" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G85" s="12" t="s">
-        <v>170</v>
+        <v>54</v>
       </c>
       <c r="H85" s="7" t="n">
         <v>1</v>
@@ -4785,7 +4660,7 @@
       </c>
       <c r="L85" s="8" t="n">
         <f aca="false">1+SUM(F85,H85,J85)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M85" s="8" t="str">
         <f aca="false">IF(L85&gt;9,"¡más de 9!","ok")</f>
@@ -4794,25 +4669,25 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C86" s="11" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D86" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E86" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F86" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G86" s="12" t="s">
-        <v>170</v>
+        <v>218</v>
       </c>
       <c r="H86" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I86" s="12"/>
       <c r="J86" s="7"/>
@@ -4821,7 +4696,7 @@
       </c>
       <c r="L86" s="8" t="n">
         <f aca="false">1+SUM(F86,H86,J86)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M86" s="8" t="str">
         <f aca="false">IF(L86&gt;9,"¡más de 9!","ok")</f>
@@ -4830,26 +4705,22 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="5" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D87" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E87" s="12" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="F87" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G87" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H87" s="7" t="n">
-        <v>3</v>
-      </c>
+      <c r="G87" s="12"/>
+      <c r="H87" s="7"/>
       <c r="I87" s="12"/>
       <c r="J87" s="7"/>
       <c r="K87" s="7" t="n">
@@ -4857,7 +4728,7 @@
       </c>
       <c r="L87" s="8" t="n">
         <f aca="false">1+SUM(F87,H87,J87)</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M87" s="8" t="str">
         <f aca="false">IF(L87&gt;9,"¡más de 9!","ok")</f>
@@ -4866,22 +4737,26 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D88" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E88" s="12" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F88" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G88" s="12"/>
-      <c r="H88" s="7"/>
+      <c r="G88" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H88" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I88" s="12"/>
       <c r="J88" s="7"/>
       <c r="K88" s="7" t="n">
@@ -4889,7 +4764,7 @@
       </c>
       <c r="L88" s="8" t="n">
         <f aca="false">1+SUM(F88,H88,J88)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M88" s="8" t="str">
         <f aca="false">IF(L88&gt;9,"¡más de 9!","ok")</f>
@@ -4898,22 +4773,22 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D89" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F89" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G89" s="12" t="s">
-        <v>222</v>
+        <v>115</v>
       </c>
       <c r="H89" s="7" t="n">
         <v>1</v>
@@ -4925,7 +4800,7 @@
       </c>
       <c r="L89" s="8" t="n">
         <f aca="false">1+SUM(F89,H89,J89)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M89" s="8" t="str">
         <f aca="false">IF(L89&gt;9,"¡más de 9!","ok")</f>
@@ -4934,22 +4809,22 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D90" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E90" s="12" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="F90" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G90" s="12" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H90" s="7" t="n">
         <v>1</v>
@@ -4970,26 +4845,22 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D91" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E91" s="12" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="F91" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G91" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="H91" s="7" t="n">
         <v>2</v>
       </c>
+      <c r="G91" s="12"/>
+      <c r="H91" s="7"/>
       <c r="I91" s="12"/>
       <c r="J91" s="7"/>
       <c r="K91" s="7" t="n">
@@ -4997,7 +4868,7 @@
       </c>
       <c r="L91" s="8" t="n">
         <f aca="false">1+SUM(F91,H91,J91)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M91" s="8" t="str">
         <f aca="false">IF(L91&gt;9,"¡más de 9!","ok")</f>
@@ -5006,25 +4877,25 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D92" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E92" s="12" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="F92" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G92" s="12" t="s">
-        <v>229</v>
+        <v>73</v>
       </c>
       <c r="H92" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I92" s="12"/>
       <c r="J92" s="7"/>
@@ -5033,7 +4904,7 @@
       </c>
       <c r="L92" s="8" t="n">
         <f aca="false">1+SUM(F92,H92,J92)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M92" s="8" t="str">
         <f aca="false">IF(L92&gt;9,"¡más de 9!","ok")</f>
@@ -5042,25 +4913,25 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D93" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E93" s="12" t="s">
-        <v>54</v>
+        <v>233</v>
       </c>
       <c r="F93" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G93" s="12" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="H93" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I93" s="12"/>
       <c r="J93" s="7"/>
@@ -5069,7 +4940,7 @@
       </c>
       <c r="L93" s="8" t="n">
         <f aca="false">1+SUM(F93,H93,J93)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M93" s="8" t="str">
         <f aca="false">IF(L93&gt;9,"¡más de 9!","ok")</f>
@@ -5078,26 +4949,22 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D94" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E94" s="12" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="F94" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G94" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="H94" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G94" s="12"/>
+      <c r="H94" s="7"/>
       <c r="I94" s="12"/>
       <c r="J94" s="7"/>
       <c r="K94" s="7" t="n">
@@ -5113,45 +4980,59 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="B95" s="10"/>
-      <c r="C95" s="10"/>
-      <c r="D95" s="10"/>
-      <c r="E95" s="10"/>
-      <c r="F95" s="10"/>
-      <c r="G95" s="10"/>
-      <c r="H95" s="10"/>
-      <c r="I95" s="10"/>
-      <c r="J95" s="10"/>
-      <c r="K95" s="10"/>
-      <c r="L95" s="10"/>
-      <c r="M95" s="10"/>
-      <c r="N95" s="10"/>
+      <c r="B95" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E95" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F95" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H95" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I95" s="12"/>
+      <c r="J95" s="7"/>
+      <c r="K95" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L95" s="8" t="n">
+        <f aca="false">1+SUM(F95,H95,J95)</f>
+        <v>3</v>
+      </c>
+      <c r="M95" s="8" t="str">
+        <f aca="false">IF(L95&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D96" s="12" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E96" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F96" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G96" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H96" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G96" s="12"/>
+      <c r="H96" s="7"/>
       <c r="I96" s="12"/>
       <c r="J96" s="7"/>
       <c r="K96" s="7" t="n">
@@ -5159,7 +5040,7 @@
       </c>
       <c r="L96" s="8" t="n">
         <f aca="false">1+SUM(F96,H96,J96)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M96" s="8" t="str">
         <f aca="false">IF(L96&gt;9,"¡más de 9!","ok")</f>
@@ -5167,50 +5048,32 @@
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B97" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="C97" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="D97" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E97" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F97" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G97" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H97" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I97" s="12"/>
-      <c r="J97" s="7"/>
-      <c r="K97" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L97" s="8" t="n">
-        <f aca="false">1+SUM(F97,H97,J97)</f>
-        <v>4</v>
-      </c>
-      <c r="M97" s="8" t="str">
-        <f aca="false">IF(L97&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="A97" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B97" s="10"/>
+      <c r="C97" s="10"/>
+      <c r="D97" s="10"/>
+      <c r="E97" s="10"/>
+      <c r="F97" s="10"/>
+      <c r="G97" s="10"/>
+      <c r="H97" s="10"/>
+      <c r="I97" s="10"/>
+      <c r="J97" s="10"/>
+      <c r="K97" s="10"/>
+      <c r="L97" s="10"/>
+      <c r="M97" s="10"/>
+      <c r="N97" s="10"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D98" s="12" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E98" s="12" t="s">
         <v>54</v>
@@ -5219,10 +5082,10 @@
         <v>1</v>
       </c>
       <c r="G98" s="12" t="s">
-        <v>170</v>
+        <v>73</v>
       </c>
       <c r="H98" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I98" s="12"/>
       <c r="J98" s="7"/>
@@ -5231,7 +5094,7 @@
       </c>
       <c r="L98" s="8" t="n">
         <f aca="false">1+SUM(F98,H98,J98)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M98" s="8" t="str">
         <f aca="false">IF(L98&gt;9,"¡más de 9!","ok")</f>
@@ -5240,13 +5103,13 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D99" s="12" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E99" s="12" t="s">
         <v>54</v>
@@ -5255,10 +5118,10 @@
         <v>1</v>
       </c>
       <c r="G99" s="12" t="s">
-        <v>170</v>
+        <v>73</v>
       </c>
       <c r="H99" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I99" s="12"/>
       <c r="J99" s="7"/>
@@ -5267,7 +5130,7 @@
       </c>
       <c r="L99" s="8" t="n">
         <f aca="false">1+SUM(F99,H99,J99)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M99" s="8" t="str">
         <f aca="false">IF(L99&gt;9,"¡más de 9!","ok")</f>
@@ -5276,13 +5139,13 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D100" s="12" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E100" s="12" t="s">
         <v>54</v>
@@ -5291,23 +5154,19 @@
         <v>1</v>
       </c>
       <c r="G100" s="12" t="s">
-        <v>170</v>
+        <v>57</v>
       </c>
       <c r="H100" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I100" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="J100" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="I100" s="12"/>
+      <c r="J100" s="7"/>
       <c r="K100" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L100" s="8" t="n">
         <f aca="false">1+SUM(F100,H100,J100)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M100" s="8" t="str">
         <f aca="false">IF(L100&gt;9,"¡más de 9!","ok")</f>
@@ -5322,7 +5181,7 @@
         <v>248</v>
       </c>
       <c r="D101" s="12" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E101" s="12" t="s">
         <v>54</v>
@@ -5334,7 +5193,7 @@
         <v>73</v>
       </c>
       <c r="H101" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I101" s="12"/>
       <c r="J101" s="7"/>
@@ -5343,7 +5202,7 @@
       </c>
       <c r="L101" s="8" t="n">
         <f aca="false">1+SUM(F101,H101,J101)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M101" s="8" t="str">
         <f aca="false">IF(L101&gt;9,"¡más de 9!","ok")</f>
@@ -5358,7 +5217,7 @@
         <v>250</v>
       </c>
       <c r="D102" s="12" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E102" s="12" t="s">
         <v>54</v>
@@ -5367,10 +5226,10 @@
         <v>1</v>
       </c>
       <c r="G102" s="12" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="H102" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I102" s="12"/>
       <c r="J102" s="7"/>
@@ -5379,7 +5238,7 @@
       </c>
       <c r="L102" s="8" t="n">
         <f aca="false">1+SUM(F102,H102,J102)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M102" s="8" t="str">
         <f aca="false">IF(L102&gt;9,"¡más de 9!","ok")</f>
@@ -5387,32 +5246,50 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="9" t="s">
+      <c r="B103" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B103" s="10"/>
-      <c r="C103" s="10"/>
-      <c r="D103" s="10"/>
-      <c r="E103" s="10"/>
-      <c r="F103" s="10"/>
-      <c r="G103" s="10"/>
-      <c r="H103" s="10"/>
-      <c r="I103" s="10"/>
-      <c r="J103" s="10"/>
-      <c r="K103" s="10"/>
-      <c r="L103" s="10"/>
-      <c r="M103" s="10"/>
-      <c r="N103" s="10"/>
+      <c r="C103" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E103" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F103" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="H103" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I103" s="12"/>
+      <c r="J103" s="7"/>
+      <c r="K103" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L103" s="8" t="n">
+        <f aca="false">1+SUM(F103,H103,J103)</f>
+        <v>3</v>
+      </c>
+      <c r="M103" s="8" t="str">
+        <f aca="false">IF(L103&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B104" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C104" s="11" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D104" s="12" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E104" s="12" t="s">
         <v>54</v>
@@ -5420,8 +5297,12 @@
       <c r="F104" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G104" s="12"/>
-      <c r="H104" s="7"/>
+      <c r="G104" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="H104" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I104" s="12"/>
       <c r="J104" s="7"/>
       <c r="K104" s="7" t="n">
@@ -5429,7 +5310,7 @@
       </c>
       <c r="L104" s="8" t="n">
         <f aca="false">1+SUM(F104,H104,J104)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M104" s="8" t="str">
         <f aca="false">IF(L104&gt;9,"¡más de 9!","ok")</f>
@@ -5438,30 +5319,38 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C105" s="11" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D105" s="12" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E105" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F105" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="H105" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I105" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="F105" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G105" s="12"/>
-      <c r="H105" s="7"/>
-      <c r="I105" s="12"/>
-      <c r="J105" s="7"/>
+      <c r="J105" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="K105" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L105" s="8" t="n">
         <f aca="false">1+SUM(F105,H105,J105)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M105" s="8" t="str">
         <f aca="false">IF(L105&gt;9,"¡más de 9!","ok")</f>
@@ -5469,59 +5358,41 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B106" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="C106" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="D106" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="E106" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F106" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G106" s="12"/>
-      <c r="H106" s="7"/>
-      <c r="I106" s="12"/>
-      <c r="J106" s="7"/>
-      <c r="K106" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L106" s="8" t="n">
-        <f aca="false">1+SUM(F106,H106,J106)</f>
-        <v>4</v>
-      </c>
-      <c r="M106" s="8" t="str">
-        <f aca="false">IF(L106&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="A106" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B106" s="10"/>
+      <c r="C106" s="10"/>
+      <c r="D106" s="10"/>
+      <c r="E106" s="10"/>
+      <c r="F106" s="10"/>
+      <c r="G106" s="10"/>
+      <c r="H106" s="10"/>
+      <c r="I106" s="10"/>
+      <c r="J106" s="10"/>
+      <c r="K106" s="10"/>
+      <c r="L106" s="10"/>
+      <c r="M106" s="10"/>
+      <c r="N106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B107" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C107" s="11" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D107" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E107" s="12" t="s">
-        <v>73</v>
+        <v>262</v>
       </c>
       <c r="F107" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G107" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="H107" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G107" s="12"/>
+      <c r="H107" s="7"/>
       <c r="I107" s="12"/>
       <c r="J107" s="7"/>
       <c r="K107" s="7" t="n">
@@ -5529,7 +5400,7 @@
       </c>
       <c r="L107" s="8" t="n">
         <f aca="false">1+SUM(F107,H107,J107)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M107" s="8" t="str">
         <f aca="false">IF(L107&gt;9,"¡más de 9!","ok")</f>
@@ -5538,26 +5409,22 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B108" s="5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C108" s="11" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D108" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E108" s="12" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F108" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G108" s="12" t="s">
-        <v>262</v>
-      </c>
-      <c r="H108" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="G108" s="12"/>
+      <c r="H108" s="7"/>
       <c r="I108" s="12"/>
       <c r="J108" s="7"/>
       <c r="K108" s="7" t="n">
@@ -5565,7 +5432,7 @@
       </c>
       <c r="L108" s="8" t="n">
         <f aca="false">1+SUM(F108,H108,J108)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M108" s="8" t="str">
         <f aca="false">IF(L108&gt;9,"¡más de 9!","ok")</f>
@@ -5574,16 +5441,16 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B109" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C109" s="11" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D109" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E109" s="12" t="s">
-        <v>69</v>
+        <v>253</v>
       </c>
       <c r="F109" s="7" t="n">
         <v>1</v>
@@ -5606,13 +5473,13 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B110" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C110" s="11" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D110" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E110" s="12" t="s">
         <v>57</v>
@@ -5620,12 +5487,8 @@
       <c r="F110" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G110" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H110" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="G110" s="12"/>
+      <c r="H110" s="7"/>
       <c r="I110" s="12"/>
       <c r="J110" s="7"/>
       <c r="K110" s="7" t="n">
@@ -5633,7 +5496,7 @@
       </c>
       <c r="L110" s="8" t="n">
         <f aca="false">1+SUM(F110,H110,J110)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M110" s="8" t="str">
         <f aca="false">IF(L110&gt;9,"¡más de 9!","ok")</f>
@@ -5642,26 +5505,22 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B111" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C111" s="11" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D111" s="12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E111" s="12" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F111" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G111" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="H111" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G111" s="12"/>
+      <c r="H111" s="7"/>
       <c r="I111" s="12"/>
       <c r="J111" s="7"/>
       <c r="K111" s="7" t="n">
@@ -5669,7 +5528,7 @@
       </c>
       <c r="L111" s="8" t="n">
         <f aca="false">1+SUM(F111,H111,J111)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M111" s="8" t="str">
         <f aca="false">IF(L111&gt;9,"¡más de 9!","ok")</f>
@@ -5677,53 +5536,35 @@
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B112" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="C112" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="D112" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="E112" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="F112" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G112" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H112" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I112" s="12"/>
-      <c r="J112" s="7"/>
-      <c r="K112" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L112" s="8" t="n">
-        <f aca="false">1+SUM(F112,H112,J112)</f>
-        <v>3</v>
-      </c>
-      <c r="M112" s="8" t="str">
-        <f aca="false">IF(L112&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="A112" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="B112" s="10"/>
+      <c r="C112" s="10"/>
+      <c r="D112" s="10"/>
+      <c r="E112" s="10"/>
+      <c r="F112" s="10"/>
+      <c r="G112" s="10"/>
+      <c r="H112" s="10"/>
+      <c r="I112" s="10"/>
+      <c r="J112" s="10"/>
+      <c r="K112" s="10"/>
+      <c r="L112" s="10"/>
+      <c r="M112" s="10"/>
+      <c r="N112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B113" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C113" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D113" s="12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E113" s="12" t="s">
-        <v>170</v>
+        <v>73</v>
       </c>
       <c r="F113" s="7" t="n">
         <v>2</v>
@@ -5746,16 +5587,16 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B114" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C114" s="11" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D114" s="12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E114" s="12" t="s">
-        <v>170</v>
+        <v>115</v>
       </c>
       <c r="F114" s="7" t="n">
         <v>1</v>
@@ -5764,7 +5605,7 @@
         <v>73</v>
       </c>
       <c r="H114" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I114" s="12"/>
       <c r="J114" s="7"/>
@@ -5773,7 +5614,7 @@
       </c>
       <c r="L114" s="8" t="n">
         <f aca="false">1+SUM(F114,H114,J114)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M114" s="8" t="str">
         <f aca="false">IF(L114&gt;9,"¡más de 9!","ok")</f>
@@ -5782,26 +5623,22 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B115" s="5" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C115" s="11" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D115" s="12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E115" s="12" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F115" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G115" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H115" s="7" t="n">
-        <v>2</v>
-      </c>
+      <c r="G115" s="12"/>
+      <c r="H115" s="7"/>
       <c r="I115" s="12"/>
       <c r="J115" s="7"/>
       <c r="K115" s="7" t="n">
@@ -5809,7 +5646,7 @@
       </c>
       <c r="L115" s="8" t="n">
         <f aca="false">1+SUM(F115,H115,J115)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M115" s="8" t="str">
         <f aca="false">IF(L115&gt;9,"¡más de 9!","ok")</f>
@@ -5818,19 +5655,19 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B116" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C116" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D116" s="12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E116" s="12" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="F116" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G116" s="12"/>
       <c r="H116" s="7"/>
@@ -5841,7 +5678,7 @@
       </c>
       <c r="L116" s="8" t="n">
         <f aca="false">1+SUM(F116,H116,J116)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M116" s="8" t="str">
         <f aca="false">IF(L116&gt;9,"¡más de 9!","ok")</f>
@@ -5850,16 +5687,16 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B117" s="5" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C117" s="11" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D117" s="12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E117" s="12" t="s">
-        <v>60</v>
+        <v>258</v>
       </c>
       <c r="F117" s="7" t="n">
         <v>1</v>
@@ -5885,77 +5722,73 @@
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B118" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="C118" s="11" t="s">
+      <c r="A118" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="D118" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="E118" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F118" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G118" s="12"/>
-      <c r="H118" s="7"/>
-      <c r="I118" s="12"/>
-      <c r="J118" s="7"/>
-      <c r="K118" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L118" s="8" t="n">
-        <f aca="false">1+SUM(F118,H118,J118)</f>
-        <v>4</v>
-      </c>
-      <c r="M118" s="8" t="str">
-        <f aca="false">IF(L118&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B118" s="10"/>
+      <c r="C118" s="10"/>
+      <c r="D118" s="10"/>
+      <c r="E118" s="10"/>
+      <c r="F118" s="10"/>
+      <c r="G118" s="10"/>
+      <c r="H118" s="10"/>
+      <c r="I118" s="10"/>
+      <c r="J118" s="10"/>
+      <c r="K118" s="10"/>
+      <c r="L118" s="10"/>
+      <c r="M118" s="10"/>
+      <c r="N118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="9" t="s">
+      <c r="B119" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="B119" s="10"/>
-      <c r="C119" s="10"/>
-      <c r="D119" s="10"/>
-      <c r="E119" s="10"/>
-      <c r="F119" s="10"/>
-      <c r="G119" s="10"/>
-      <c r="H119" s="10"/>
-      <c r="I119" s="10"/>
-      <c r="J119" s="10"/>
-      <c r="K119" s="10"/>
-      <c r="L119" s="10"/>
-      <c r="M119" s="10"/>
-      <c r="N119" s="10"/>
+      <c r="C119" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="D119" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E119" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F119" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G119" s="12"/>
+      <c r="H119" s="7"/>
+      <c r="I119" s="12"/>
+      <c r="J119" s="7"/>
+      <c r="K119" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L119" s="8" t="n">
+        <f aca="false">1+SUM(F119,H119,J119)</f>
+        <v>2</v>
+      </c>
+      <c r="M119" s="8" t="str">
+        <f aca="false">IF(L119&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C120" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D120" s="12" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E120" s="12" t="s">
-        <v>54</v>
+        <v>288</v>
       </c>
       <c r="F120" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G120" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H120" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="G120" s="12"/>
+      <c r="H120" s="7"/>
       <c r="I120" s="12"/>
       <c r="J120" s="7"/>
       <c r="K120" s="7" t="n">
@@ -5963,7 +5796,7 @@
       </c>
       <c r="L120" s="8" t="n">
         <f aca="false">1+SUM(F120,H120,J120)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M120" s="8" t="str">
         <f aca="false">IF(L120&gt;9,"¡más de 9!","ok")</f>
@@ -5972,26 +5805,22 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C121" s="11" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D121" s="12" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E121" s="12" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="F121" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G121" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H121" s="7" t="n">
         <v>2</v>
       </c>
+      <c r="G121" s="12"/>
+      <c r="H121" s="7"/>
       <c r="I121" s="12"/>
       <c r="J121" s="7"/>
       <c r="K121" s="7" t="n">
@@ -5999,7 +5828,7 @@
       </c>
       <c r="L121" s="8" t="n">
         <f aca="false">1+SUM(F121,H121,J121)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M121" s="8" t="str">
         <f aca="false">IF(L121&gt;9,"¡más de 9!","ok")</f>
@@ -6008,26 +5837,22 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C122" s="11" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D122" s="12" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E122" s="12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F122" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G122" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="H122" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G122" s="12"/>
+      <c r="H122" s="7"/>
       <c r="I122" s="12"/>
       <c r="J122" s="7"/>
       <c r="K122" s="7" t="n">
@@ -6044,25 +5869,25 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C123" s="11" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D123" s="12" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="E123" s="12" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="F123" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G123" s="12" t="s">
-        <v>73</v>
+        <v>150</v>
       </c>
       <c r="H123" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I123" s="12"/>
       <c r="J123" s="7"/>
@@ -6071,734 +5896,45 @@
       </c>
       <c r="L123" s="8" t="n">
         <f aca="false">1+SUM(F123,H123,J123)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M123" s="8" t="str">
         <f aca="false">IF(L123&gt;9,"¡más de 9!","ok")</f>
         <v>ok</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B124" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="C124" s="11" t="s">
-        <v>294</v>
-      </c>
-      <c r="D124" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E124" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F124" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G124" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H124" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I124" s="12"/>
-      <c r="J124" s="7"/>
-      <c r="K124" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L124" s="8" t="n">
-        <f aca="false">1+SUM(F124,H124,J124)</f>
-        <v>3</v>
-      </c>
-      <c r="M124" s="8" t="str">
-        <f aca="false">IF(L124&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B125" s="5" t="s">
+      <c r="A125" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="C125" s="11" t="s">
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="D125" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E125" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F125" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G125" s="12" t="s">
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="H125" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I125" s="12"/>
-      <c r="J125" s="7"/>
-      <c r="K125" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L125" s="8" t="n">
-        <f aca="false">1+SUM(F125,H125,J125)</f>
-        <v>3</v>
-      </c>
-      <c r="M125" s="8" t="str">
-        <f aca="false">IF(L125&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B126" s="5" t="s">
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="5" t="s">
         <v>298</v>
-      </c>
-      <c r="C126" s="11" t="s">
-        <v>299</v>
-      </c>
-      <c r="D126" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E126" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F126" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G126" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="H126" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I126" s="12"/>
-      <c r="J126" s="7"/>
-      <c r="K126" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L126" s="8" t="n">
-        <f aca="false">1+SUM(F126,H126,J126)</f>
-        <v>3</v>
-      </c>
-      <c r="M126" s="8" t="str">
-        <f aca="false">IF(L126&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B127" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="C127" s="11" t="s">
-        <v>301</v>
-      </c>
-      <c r="D127" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="E127" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F127" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G127" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="H127" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I127" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="J127" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="K127" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L127" s="8" t="n">
-        <f aca="false">1+SUM(F127,H127,J127)</f>
-        <v>5</v>
-      </c>
-      <c r="M127" s="8" t="str">
-        <f aca="false">IF(L127&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="B128" s="10"/>
-      <c r="C128" s="10"/>
-      <c r="D128" s="10"/>
-      <c r="E128" s="10"/>
-      <c r="F128" s="10"/>
-      <c r="G128" s="10"/>
-      <c r="H128" s="10"/>
-      <c r="I128" s="10"/>
-      <c r="J128" s="10"/>
-      <c r="K128" s="10"/>
-      <c r="L128" s="10"/>
-      <c r="M128" s="10"/>
-      <c r="N128" s="10"/>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="C129" s="11" t="s">
-        <v>305</v>
-      </c>
-      <c r="D129" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E129" s="12" t="s">
-        <v>306</v>
-      </c>
-      <c r="F129" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G129" s="12"/>
-      <c r="H129" s="7"/>
-      <c r="I129" s="12"/>
-      <c r="J129" s="7"/>
-      <c r="K129" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L129" s="8" t="n">
-        <f aca="false">1+SUM(F129,H129,J129)</f>
-        <v>2</v>
-      </c>
-      <c r="M129" s="8" t="str">
-        <f aca="false">IF(L129&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B130" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="C130" s="11" t="s">
-        <v>308</v>
-      </c>
-      <c r="D130" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E130" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="F130" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G130" s="12"/>
-      <c r="H130" s="7"/>
-      <c r="I130" s="12"/>
-      <c r="J130" s="7"/>
-      <c r="K130" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L130" s="8" t="n">
-        <f aca="false">1+SUM(F130,H130,J130)</f>
-        <v>2</v>
-      </c>
-      <c r="M130" s="8" t="str">
-        <f aca="false">IF(L130&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B131" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="C131" s="11" t="s">
-        <v>310</v>
-      </c>
-      <c r="D131" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E131" s="12" t="s">
-        <v>297</v>
-      </c>
-      <c r="F131" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G131" s="12"/>
-      <c r="H131" s="7"/>
-      <c r="I131" s="12"/>
-      <c r="J131" s="7"/>
-      <c r="K131" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L131" s="8" t="n">
-        <f aca="false">1+SUM(F131,H131,J131)</f>
-        <v>2</v>
-      </c>
-      <c r="M131" s="8" t="str">
-        <f aca="false">IF(L131&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B132" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="C132" s="11" t="s">
-        <v>312</v>
-      </c>
-      <c r="D132" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E132" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="F132" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G132" s="12"/>
-      <c r="H132" s="7"/>
-      <c r="I132" s="12"/>
-      <c r="J132" s="7"/>
-      <c r="K132" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L132" s="8" t="n">
-        <f aca="false">1+SUM(F132,H132,J132)</f>
-        <v>2</v>
-      </c>
-      <c r="M132" s="8" t="str">
-        <f aca="false">IF(L132&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B133" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="C133" s="11" t="s">
-        <v>314</v>
-      </c>
-      <c r="D133" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E133" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="F133" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G133" s="12"/>
-      <c r="H133" s="7"/>
-      <c r="I133" s="12"/>
-      <c r="J133" s="7"/>
-      <c r="K133" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L133" s="8" t="n">
-        <f aca="false">1+SUM(F133,H133,J133)</f>
-        <v>2</v>
-      </c>
-      <c r="M133" s="8" t="str">
-        <f aca="false">IF(L133&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="B134" s="10"/>
-      <c r="C134" s="10"/>
-      <c r="D134" s="10"/>
-      <c r="E134" s="10"/>
-      <c r="F134" s="10"/>
-      <c r="G134" s="10"/>
-      <c r="H134" s="10"/>
-      <c r="I134" s="10"/>
-      <c r="J134" s="10"/>
-      <c r="K134" s="10"/>
-      <c r="L134" s="10"/>
-      <c r="M134" s="10"/>
-      <c r="N134" s="10"/>
-    </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B135" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="C135" s="11" t="s">
-        <v>317</v>
-      </c>
-      <c r="D135" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E135" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F135" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G135" s="12"/>
-      <c r="H135" s="7"/>
-      <c r="I135" s="12"/>
-      <c r="J135" s="7"/>
-      <c r="K135" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L135" s="8" t="n">
-        <f aca="false">1+SUM(F135,H135,J135)</f>
-        <v>3</v>
-      </c>
-      <c r="M135" s="8" t="str">
-        <f aca="false">IF(L135&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B136" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="C136" s="11" t="s">
-        <v>319</v>
-      </c>
-      <c r="D136" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E136" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F136" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G136" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H136" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I136" s="12"/>
-      <c r="J136" s="7"/>
-      <c r="K136" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L136" s="8" t="n">
-        <f aca="false">1+SUM(F136,H136,J136)</f>
-        <v>3</v>
-      </c>
-      <c r="M136" s="8" t="str">
-        <f aca="false">IF(L136&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B137" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="C137" s="11" t="s">
-        <v>321</v>
-      </c>
-      <c r="D137" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E137" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="F137" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G137" s="12"/>
-      <c r="H137" s="7"/>
-      <c r="I137" s="12"/>
-      <c r="J137" s="7"/>
-      <c r="K137" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L137" s="8" t="n">
-        <f aca="false">1+SUM(F137,H137,J137)</f>
-        <v>2</v>
-      </c>
-      <c r="M137" s="8" t="str">
-        <f aca="false">IF(L137&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B138" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="C138" s="11" t="s">
-        <v>324</v>
-      </c>
-      <c r="D138" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E138" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="F138" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G138" s="12"/>
-      <c r="H138" s="7"/>
-      <c r="I138" s="12"/>
-      <c r="J138" s="7"/>
-      <c r="K138" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L138" s="8" t="n">
-        <f aca="false">1+SUM(F138,H138,J138)</f>
-        <v>2</v>
-      </c>
-      <c r="M138" s="8" t="str">
-        <f aca="false">IF(L138&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B139" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C139" s="11" t="s">
-        <v>326</v>
-      </c>
-      <c r="D139" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E139" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="F139" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G139" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H139" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I139" s="12"/>
-      <c r="J139" s="7"/>
-      <c r="K139" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L139" s="8" t="n">
-        <f aca="false">1+SUM(F139,H139,J139)</f>
-        <v>3</v>
-      </c>
-      <c r="M139" s="8" t="str">
-        <f aca="false">IF(L139&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="9" t="s">
-        <v>327</v>
-      </c>
-      <c r="B140" s="10"/>
-      <c r="C140" s="10"/>
-      <c r="D140" s="10"/>
-      <c r="E140" s="10"/>
-      <c r="F140" s="10"/>
-      <c r="G140" s="10"/>
-      <c r="H140" s="10"/>
-      <c r="I140" s="10"/>
-      <c r="J140" s="10"/>
-      <c r="K140" s="10"/>
-      <c r="L140" s="10"/>
-      <c r="M140" s="10"/>
-      <c r="N140" s="10"/>
-    </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B141" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="C141" s="11" t="s">
-        <v>329</v>
-      </c>
-      <c r="D141" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E141" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="F141" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G141" s="12"/>
-      <c r="H141" s="7"/>
-      <c r="I141" s="12"/>
-      <c r="J141" s="7"/>
-      <c r="K141" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L141" s="8" t="n">
-        <f aca="false">1+SUM(F141,H141,J141)</f>
-        <v>2</v>
-      </c>
-      <c r="M141" s="8" t="str">
-        <f aca="false">IF(L141&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B142" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="C142" s="11" t="s">
-        <v>331</v>
-      </c>
-      <c r="D142" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E142" s="12" t="s">
-        <v>332</v>
-      </c>
-      <c r="F142" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G142" s="12"/>
-      <c r="H142" s="7"/>
-      <c r="I142" s="12"/>
-      <c r="J142" s="7"/>
-      <c r="K142" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L142" s="8" t="n">
-        <f aca="false">1+SUM(F142,H142,J142)</f>
-        <v>2</v>
-      </c>
-      <c r="M142" s="8" t="str">
-        <f aca="false">IF(L142&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B143" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="C143" s="11" t="s">
-        <v>334</v>
-      </c>
-      <c r="D143" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E143" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="F143" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G143" s="12"/>
-      <c r="H143" s="7"/>
-      <c r="I143" s="12"/>
-      <c r="J143" s="7"/>
-      <c r="K143" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L143" s="8" t="n">
-        <f aca="false">1+SUM(F143,H143,J143)</f>
-        <v>3</v>
-      </c>
-      <c r="M143" s="8" t="str">
-        <f aca="false">IF(L143&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B144" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="C144" s="11" t="s">
-        <v>336</v>
-      </c>
-      <c r="D144" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E144" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F144" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G144" s="12"/>
-      <c r="H144" s="7"/>
-      <c r="I144" s="12"/>
-      <c r="J144" s="7"/>
-      <c r="K144" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L144" s="8" t="n">
-        <f aca="false">1+SUM(F144,H144,J144)</f>
-        <v>3</v>
-      </c>
-      <c r="M144" s="8" t="str">
-        <f aca="false">IF(L144&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B145" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="C145" s="11" t="s">
-        <v>338</v>
-      </c>
-      <c r="D145" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E145" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="F145" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G145" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H145" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I145" s="12"/>
-      <c r="J145" s="7"/>
-      <c r="K145" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L145" s="8" t="n">
-        <f aca="false">1+SUM(F145,H145,J145)</f>
-        <v>3</v>
-      </c>
-      <c r="M145" s="8" t="str">
-        <f aca="false">IF(L145&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
-    </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="5" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="5" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="5" t="s">
-        <v>341</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E145 G5:G145 I5:I145" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E123 G5:G123 I5:I123" type="list">
       <formula1>Leyenda!$A$5:$A$60</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D145" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D5:D123" type="list">
       <formula1>Leyenda!$D$5:$D$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6828,21 +5964,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>342</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>343</v>
+        <v>300</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>344</v>
+        <v>301</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>345</v>
+        <v>302</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>346</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6850,10 +5986,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>347</v>
+        <v>304</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>348</v>
+        <v>305</v>
       </c>
       <c r="D4" s="15"/>
     </row>
@@ -6862,10 +5998,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>349</v>
+        <v>306</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>350</v>
+        <v>307</v>
       </c>
       <c r="D5" s="15"/>
     </row>
@@ -6874,10 +6010,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>351</v>
+        <v>308</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>352</v>
+        <v>309</v>
       </c>
       <c r="D6" s="15"/>
     </row>
@@ -6886,10 +6022,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>353</v>
+        <v>310</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>354</v>
+        <v>311</v>
       </c>
       <c r="D7" s="15"/>
     </row>
@@ -6898,10 +6034,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>355</v>
+        <v>312</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>356</v>
+        <v>313</v>
       </c>
       <c r="D8" s="15"/>
     </row>
@@ -6910,10 +6046,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>357</v>
+        <v>314</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>358</v>
+        <v>315</v>
       </c>
       <c r="D9" s="15"/>
     </row>
@@ -6944,26 +6080,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>359</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>360</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>361</v>
+        <v>318</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>43</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>362</v>
+        <v>319</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>363</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6971,7 +6107,7 @@
         <v>73</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>364</v>
+        <v>321</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>17</v>
@@ -6988,7 +6124,7 @@
         <v>54</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>365</v>
+        <v>322</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>23</v>
@@ -6997,15 +6133,15 @@
         <v>20</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>366</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>367</v>
+        <v>324</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>28</v>
@@ -7022,7 +6158,7 @@
         <v>60</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>368</v>
+        <v>325</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>31</v>
@@ -7036,10 +6172,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>222</v>
+        <v>186</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>369</v>
+        <v>326</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>34</v>
@@ -7056,53 +6192,53 @@
         <v>69</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>370</v>
+        <v>327</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>36</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>371</v>
+        <v>328</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>372</v>
+        <v>329</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>229</v>
+        <v>193</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>373</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>306</v>
+        <v>262</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>374</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>246</v>
+        <v>206</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>375</v>
+        <v>332</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7110,55 +6246,55 @@
         <v>66</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>376</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>297</v>
+        <v>253</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>377</v>
+        <v>334</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>277</v>
+        <v>233</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>302</v>
+        <v>258</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>379</v>
+        <v>336</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>322</v>
+        <v>278</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>380</v>
+        <v>337</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>381</v>
+        <v>338</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>332</v>
+        <v>288</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>382</v>
+        <v>339</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7166,7 +6302,7 @@
         <v>57</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>383</v>
+        <v>340</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7174,23 +6310,23 @@
         <v>63</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>384</v>
+        <v>341</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>262</v>
+        <v>218</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>385</v>
+        <v>342</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>386</v>
+        <v>343</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7198,15 +6334,15 @@
         <v>14</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>387</v>
+        <v>344</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>366</v>
+        <v>323</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>388</v>
+        <v>345</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7214,7 +6350,7 @@
         <v>15</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>389</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ruedos unificados: redondeado y cola como moldes de ruedo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5ByHgyXpZwXMUmHLQD8vD
</commit_message>
<xml_diff>
--- a/docs/recetas_moldes_propuesta.xlsx
+++ b/docs/recetas_moldes_propuesta.xlsx
@@ -349,6 +349,18 @@
     <t xml:space="preserve">modamod:molde_ruedo_pico</t>
   </si>
   <si>
+    <t xml:space="preserve">Molde de Ruedo: Redondeado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modamod:molde_ruedo_redondeado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molde de Ruedo: Con cola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modamod:molde_ruedo_cola</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pollera</t>
   </si>
   <si>
@@ -443,18 +455,6 @@
   </si>
   <si>
     <t xml:space="preserve">Capa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molde de Capa: Ruedo redondeado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_ruedo_redondeado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Molde de Capa: Ruedo con cola</t>
-  </si>
-  <si>
-    <t xml:space="preserve">modamod:molde_capa_ruedo_cola</t>
   </si>
   <si>
     <t xml:space="preserve">Molde de Capa: Cuello alto</t>
@@ -2828,29 +2828,47 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
+      <c r="B31" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="10"/>
-      <c r="N31" s="10"/>
+      <c r="C31" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="12"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" s="8" t="n">
+        <f aca="false">1+SUM(F31,H31,J31)</f>
+        <v>3</v>
+      </c>
+      <c r="M31" s="8" t="str">
+        <f aca="false">IF(L31&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>17</v>
@@ -2882,40 +2900,22 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C33" s="11" t="s">
+      <c r="A33" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D33" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I33" s="12"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" s="8" t="n">
-        <f aca="false">1+SUM(F33,H33,J33)</f>
-        <v>3</v>
-      </c>
-      <c r="M33" s="8" t="str">
-        <f aca="false">IF(L33&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
+      <c r="L33" s="10"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="5" t="s">
@@ -2937,20 +2937,16 @@
         <v>60</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I34" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="J34" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I34" s="12"/>
+      <c r="J34" s="7"/>
       <c r="K34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L34" s="8" t="n">
         <f aca="false">1+SUM(F34,H34,J34)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M34" s="8" t="str">
         <f aca="false">IF(L34&gt;9,"¡más de 9!","ok")</f>
@@ -2959,11 +2955,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C35" s="11" t="s">
-        <v>117</v>
-      </c>
       <c r="D35" s="12" t="s">
         <v>17</v>
       </c>
@@ -2974,23 +2970,19 @@
         <v>1</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I35" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="J35" s="7" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I35" s="12"/>
+      <c r="J35" s="7"/>
       <c r="K35" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L35" s="8" t="n">
         <f aca="false">1+SUM(F35,H35,J35)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M35" s="8" t="str">
         <f aca="false">IF(L35&gt;9,"¡más de 9!","ok")</f>
@@ -2999,28 +2991,32 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="D36" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="D36" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H36" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I36" s="12"/>
-      <c r="J36" s="7"/>
+      <c r="J36" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K36" s="7" t="n">
         <v>1</v>
       </c>
@@ -3050,13 +3046,13 @@
         <v>1</v>
       </c>
       <c r="G37" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I37" s="12" t="s">
         <v>73</v>
-      </c>
-      <c r="H37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I37" s="12" t="s">
-        <v>60</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>1</v>
@@ -3066,7 +3062,7 @@
       </c>
       <c r="L37" s="8" t="n">
         <f aca="false">1+SUM(F37,H37,J37)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M37" s="8" t="str">
         <f aca="false">IF(L37&gt;9,"¡más de 9!","ok")</f>
@@ -3074,29 +3070,47 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9" t="s">
+      <c r="B38" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
+      <c r="C38" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" s="12"/>
+      <c r="J38" s="7"/>
+      <c r="K38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" s="8" t="n">
+        <f aca="false">1+SUM(F38,H38,J38)</f>
+        <v>4</v>
+      </c>
+      <c r="M38" s="8" t="str">
+        <f aca="false">IF(L38&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>17</v>
@@ -3113,14 +3127,18 @@
       <c r="H39" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="I39" s="12"/>
-      <c r="J39" s="7"/>
+      <c r="I39" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="K39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="L39" s="8" t="n">
         <f aca="false">1+SUM(F39,H39,J39)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M39" s="8" t="str">
         <f aca="false">IF(L39&gt;9,"¡más de 9!","ok")</f>
@@ -3128,40 +3146,22 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C40" s="11" t="s">
+      <c r="A40" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D40" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E40" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="H40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I40" s="12"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L40" s="8" t="n">
-        <f aca="false">1+SUM(F40,H40,J40)</f>
-        <v>3</v>
-      </c>
-      <c r="M40" s="8" t="str">
-        <f aca="false">IF(L40&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="5" t="s">
@@ -3180,7 +3180,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>1</v>
@@ -3216,7 +3216,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="H42" s="7" t="n">
         <v>1</v>
@@ -3252,7 +3252,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="H43" s="7" t="n">
         <v>1</v>
@@ -3288,10 +3288,10 @@
         <v>1</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>73</v>
+        <v>105</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I44" s="12"/>
       <c r="J44" s="7"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="L44" s="8" t="n">
         <f aca="false">1+SUM(F44,H44,J44)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M44" s="8" t="str">
         <f aca="false">IF(L44&gt;9,"¡más de 9!","ok")</f>
@@ -3323,8 +3323,12 @@
       <c r="F45" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G45" s="12"/>
-      <c r="H45" s="7"/>
+      <c r="G45" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H45" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I45" s="12"/>
       <c r="J45" s="7"/>
       <c r="K45" s="7" t="n">
@@ -3332,7 +3336,7 @@
       </c>
       <c r="L45" s="8" t="n">
         <f aca="false">1+SUM(F45,H45,J45)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M45" s="8" t="str">
         <f aca="false">IF(L45&gt;9,"¡más de 9!","ok")</f>
@@ -3359,7 +3363,7 @@
         <v>73</v>
       </c>
       <c r="H46" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I46" s="12"/>
       <c r="J46" s="7"/>
@@ -3368,7 +3372,7 @@
       </c>
       <c r="L46" s="8" t="n">
         <f aca="false">1+SUM(F46,H46,J46)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M46" s="8" t="str">
         <f aca="false">IF(L46&gt;9,"¡más de 9!","ok")</f>
@@ -3376,29 +3380,43 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="9" t="s">
+      <c r="B47" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
-      <c r="I47" s="10"/>
-      <c r="J47" s="10"/>
-      <c r="K47" s="10"/>
-      <c r="L47" s="10"/>
-      <c r="M47" s="10"/>
-      <c r="N47" s="10"/>
+      <c r="C47" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="12"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="12"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" s="8" t="n">
+        <f aca="false">1+SUM(F47,H47,J47)</f>
+        <v>2</v>
+      </c>
+      <c r="M47" s="8" t="str">
+        <f aca="false">IF(L47&gt;9,"¡más de 9!","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D48" s="12" t="s">
         <v>17</v>
@@ -3430,40 +3448,22 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C49" s="11" t="s">
+      <c r="A49" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="D49" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="H49" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="I49" s="12"/>
-      <c r="J49" s="7"/>
-      <c r="K49" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L49" s="8" t="n">
-        <f aca="false">1+SUM(F49,H49,J49)</f>
-        <v>5</v>
-      </c>
-      <c r="M49" s="8" t="str">
-        <f aca="false">IF(L49&gt;9,"¡más de 9!","ok")</f>
-        <v>ok</v>
-      </c>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
+      <c r="L49" s="10"/>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="5" t="s">
@@ -4788,7 +4788,7 @@
         <v>2</v>
       </c>
       <c r="G89" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H89" s="7" t="n">
         <v>1</v>
@@ -5596,7 +5596,7 @@
         <v>34</v>
       </c>
       <c r="E114" s="12" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F114" s="7" t="n">
         <v>1</v>
@@ -6283,7 +6283,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>338</v>

</xml_diff>